<commit_message>
Fix Facebook Marketplace bulk template validation errors
Use exact VALIDATION condition strings and a required category
from the dropdown list so the upload file passes spreadsheet checks.

Co-authored-by: SEAS2025 <SEAS2025@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/exports/facebook-ambulances-marketplace-bulk-UPLOAD.xlsx
+++ b/public/exports/facebook-ambulances-marketplace-bulk-UPLOAD.xlsx
@@ -561,7 +561,7 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>2008 Ford E-350 Diesel Ambulance Not Running Project/Parts $1500</t>
+          <t>2008 Ford E-350 Diesel Ambulance Not Running Project/Parts</t>
         </is>
       </c>
       <c r="B5" s="0" t="n">
@@ -569,38 +569,42 @@
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>Used - Fair</t>
+          <t>Used – fair</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>FOR SALE: 2008 Ford E-350 Super Duty diesel Type II ambulance — Truck 1.
+          <t>FOR SALE: 2008 Ford E-350 Super Duty diesel Type II ambulance - Truck 1.
 IMPORTANT: This vehicle DOES NOT RUN. Sold as a non-running project, parts donor, or ambulance body only. Not roadworthy. Sold as-is, where-is, with no warranty.
 VIN: 1FDSS34P88DA70177
 License: 5525PN
 Odometer: 365,027 miles
 Title status: Salvage (confirm at pickup)
 Details:
-• 6.0L V8 diesel
-• New transmission installed at 347,847 miles (2023)
-• Headlights replaced; new tires and brakes
-• Outdoor-stored retired fleet unit
-• No medical equipment, drugs, or patient-care supplies included
-Price: $1,500 (firm unless otherwise agreed)
+- 6.0L V8 diesel
+- New transmission installed at 347,847 miles (2023)
+- Headlights replaced; new tires and brakes
+- Outdoor-stored retired fleet unit
+- No medical equipment, drugs, or patient-care supplies included
+Price: $1,500
 Local pickup only: 200 Louthian Way, Blythewood, SC 29016
 Buyer arranges and pays for all towing/transport.
 Seller: Prince George Transport (licensed SC non-emergency ambulance service).
 Call/text: (803) 231-9420
-Please confirm VIN, title, and mileage in person before paying.
-Serious local buyers only. No shipping of the vehicle by seller.</t>
-        </is>
-      </c>
-      <c r="E5" s="0" t="n"/>
+Confirm VIN, title, and mileage in person before paying.
+Serious local buyers only.</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>Auto Parts &amp; Accessories//Car Parts &amp; Accessories</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2008 Ford E-350 Diesel Ambulance Not Running Project/Parts $1500</t>
+          <t>2008 Ford E-350 Diesel Ambulance Not Running Project/Parts</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -608,36 +612,41 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Used - Fair</t>
+          <t>Used – fair</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>FOR SALE: 2008 Ford E-350 Super Duty diesel Type II ambulance — Truck 2.
+          <t>FOR SALE: 2008 Ford E-350 Super Duty diesel Type II ambulance - Truck 2.
 IMPORTANT: This vehicle DOES NOT RUN. Sold as a non-running project, parts donor, or ambulance body only. Not roadworthy. Sold as-is, where-is, with no warranty.
 VIN: 1FDSS34P58DB04415
 License: SS25PN
 Odometer: 176,487 miles
 Title status: Salvage (confirm at pickup)
 Details:
-• Diesel
-• Injectors replaced in 2023
-• Outdoor-stored retired fleet unit
-• No medical equipment, drugs, or patient-care supplies included
-Price: $1,500 (firm unless otherwise agreed)
+- Diesel
+- Injectors replaced in 2023
+- Outdoor-stored retired fleet unit
+- No medical equipment, drugs, or patient-care supplies included
+Price: $1,500
 Local pickup only: 200 Louthian Way, Blythewood, SC 29016
 Buyer arranges and pays for all towing/transport.
 Seller: Prince George Transport (licensed SC non-emergency ambulance service).
 Call/text: (803) 231-9420
-Please confirm VIN, title, and mileage in person before paying.
-Serious local buyers only. No shipping of the vehicle by seller.</t>
+Confirm VIN, title, and mileage in person before paying.
+Serious local buyers only.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Auto Parts &amp; Accessories//Car Parts &amp; Accessories</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2010 Ford E-350 Diesel Ambulance Not Running Project/Parts $1500</t>
+          <t>2010 Ford E-350 Diesel Ambulance Not Running Project/Parts</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -645,34 +654,39 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Used - Fair</t>
+          <t>Used – fair</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>FOR SALE: 2010 Ford E-350 Super Duty diesel Type II ambulance — Truck 3.
+          <t>FOR SALE: 2010 Ford E-350 Super Duty diesel Type II ambulance - Truck 3.
 IMPORTANT: This vehicle DOES NOT RUN. Sold as a non-running project, parts donor, or ambulance body only. Not roadworthy. Sold as-is, where-is, with no warranty.
 VIN: 1FDSS3EPADA25619
 Odometer: 355,825 miles
 Title status: Salvage (confirm at pickup)
 Details:
-• Diesel
-• Outdoor-stored retired fleet unit
-• No medical equipment, drugs, or patient-care supplies included
-Price: $1,500 (firm unless otherwise agreed)
+- Diesel
+- Outdoor-stored retired fleet unit
+- No medical equipment, drugs, or patient-care supplies included
+Price: $1,500
 Local pickup only: 200 Louthian Way, Blythewood, SC 29016
 Buyer arranges and pays for all towing/transport.
 Seller: Prince George Transport (licensed SC non-emergency ambulance service).
 Call/text: (803) 231-9420
-Please confirm VIN, title, and mileage in person before paying.
-Serious local buyers only. No shipping of the vehicle by seller.</t>
+Confirm VIN, title, and mileage in person before paying.
+Serious local buyers only.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Auto Parts &amp; Accessories//Car Parts &amp; Accessories</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2009 Ford E-350 Diesel Ambulance Not Running Project/Parts $1500</t>
+          <t>2009 Ford E-350 Diesel Ambulance Not Running Project/Parts</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -680,35 +694,40 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Used - Fair</t>
+          <t>Used – fair</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>FOR SALE: 2009 Ford E-350 Super Duty diesel Type II ambulance — Truck 4.
+          <t>FOR SALE: 2009 Ford E-350 Super Duty diesel Type II ambulance - Truck 4.
 IMPORTANT: This vehicle DOES NOT RUN. Sold as a non-running project, parts donor, or ambulance body only. Not roadworthy. Sold as-is, where-is, with no warranty.
 VIN: 1FDSSES2ADA88103
 Odometer: 346,618 miles
 Title status: Salvage (confirm at pickup)
 Details:
-• Diesel
-• Refurbished AC — condition unknown
-• Outdoor-stored retired fleet unit
-• No medical equipment, drugs, or patient-care supplies included
-Price: $1,500 (firm unless otherwise agreed)
+- Diesel
+- Refurbished AC - condition unknown
+- Outdoor-stored retired fleet unit
+- No medical equipment, drugs, or patient-care supplies included
+Price: $1,500
 Local pickup only: 200 Louthian Way, Blythewood, SC 29016
 Buyer arranges and pays for all towing/transport.
 Seller: Prince George Transport (licensed SC non-emergency ambulance service).
 Call/text: (803) 231-9420
-Please confirm VIN, title, and mileage in person before paying.
-Serious local buyers only. No shipping of the vehicle by seller.</t>
+Confirm VIN, title, and mileage in person before paying.
+Serious local buyers only.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Auto Parts &amp; Accessories//Car Parts &amp; Accessories</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2010 Ford E-350 Diesel Ambulance Not Running Project/Parts $1500</t>
+          <t>2010 Ford E-350 Diesel Ambulance Not Running Project/Parts</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -716,27 +735,32 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Used - Fair</t>
+          <t>Used – fair</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>FOR SALE: 2010 Ford E-350 Super Duty diesel Type II ambulance — Truck 5.
+          <t>FOR SALE: 2010 Ford E-350 Super Duty diesel Type II ambulance - Truck 5.
 IMPORTANT: This vehicle DOES NOT RUN. Sold as a non-running project, parts donor, or ambulance body only. Not roadworthy. Sold as-is, where-is, with no warranty.
 VIN: 1FDSSEP7ADA03185
 Odometer: 377,409 miles
 Title status: Salvage (confirm at pickup)
 Details:
-• Diesel
-• Outdoor-stored retired fleet unit
-• No medical equipment, drugs, or patient-care supplies included
-Price: $1,500 (firm unless otherwise agreed)
+- Diesel
+- Outdoor-stored retired fleet unit
+- No medical equipment, drugs, or patient-care supplies included
+Price: $1,500
 Local pickup only: 200 Louthian Way, Blythewood, SC 29016
 Buyer arranges and pays for all towing/transport.
 Seller: Prince George Transport (licensed SC non-emergency ambulance service).
 Call/text: (803) 231-9420
-Please confirm VIN, title, and mileage in person before paying.
-Serious local buyers only. No shipping of the vehicle by seller.</t>
+Confirm VIN, title, and mileage in person before paying.
+Serious local buyers only.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Auto Parts &amp; Accessories//Car Parts &amp; Accessories</t>
         </is>
       </c>
     </row>

</xml_diff>